<commit_message>
feat: implement expense page with charts, filters, CRUD operations and export functionality
</commit_message>
<xml_diff>
--- a/backend/expense_details.xlsx
+++ b/backend/expense_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,35 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Fast Food</v>
+        <v>Medicine</v>
       </c>
       <c r="B2">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="C2" t="str">
-        <v>Food</v>
+        <v>Healthcare</v>
       </c>
       <c r="D2" t="str">
-        <v>2/9/2026</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Snacks</v>
-      </c>
-      <c r="B3">
-        <v>1700</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Food</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2/9/2026</v>
+        <v>3/17/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement profile page functionality with update profile, change password and logout logic
</commit_message>
<xml_diff>
--- a/backend/expense_details.xlsx
+++ b/backend/expense_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,9 +427,37 @@
         <v>3/17/2026</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Fast Food</v>
+      </c>
+      <c r="B3">
+        <v>1500</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Food</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2/9/2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Snacks</v>
+      </c>
+      <c r="B4">
+        <v>1700</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Food</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2/9/2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>